<commit_message>
chore: 2 bug fixed, e2e 8/8, regen
</commit_message>
<xml_diff>
--- a/reports/Shiftbase-QA-Report.xlsx
+++ b/reports/Shiftbase-QA-Report.xlsx
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -2962,7 +2962,11 @@
           <t>Dropdown reload otomatis setelah import sukses</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Reload employees setelah import sukses (Attendance.tsx)</t>
+        </is>
+      </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
           <t>TC-WEB-05</t>
@@ -2987,7 +2991,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -3006,7 +3010,11 @@
           <t>Tetap di tab Absensi (persist state/route)</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Persist tab di localStorage (App.tsx Shell)</t>
+        </is>
+      </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
           <t>TC-WEB-05</t>

</xml_diff>